<commit_message>
Newstead Rev G: referee swap, Langtrees credit, Sunny Lotay core team
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RKGFyarCMuMinKYL7AiBap
</commit_message>
<xml_diff>
--- a/FP/VP527277/Final/JCE_CostSheet_VP527277_RevG.xlsx
+++ b/FP/VP527277/Final/JCE_CostSheet_VP527277_RevG.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H55"/>
+  <dimension ref="A1:H56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="2" max="2"/>
@@ -1673,7 +1673,7 @@
       <c r="A42" t="inlineStr"/>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Equipment and travel [TBC - Jayden: rates]</t>
+          <t>Equipment, travel and associate certifying engineer [TBC - Jayden: rates]</t>
         </is>
       </c>
       <c r="C42" t="inlineStr"/>
@@ -1741,72 +1741,63 @@
         <v>3080</v>
       </c>
     </row>
-    <row r="48">
-      <c r="A48" s="1" t="inlineStr">
+    <row r="47">
+      <c r="A47" t="inlineStr"/>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>Associate certifying engineer (Sunny Lotay, Lotay Civil): independent technical review and certification of JCE reports, 24 h at $220/h allowance (cost plus 10%) [TBC - Jayden to confirm rate]</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr"/>
+      <c r="D47" t="inlineStr"/>
+      <c r="E47" t="inlineStr"/>
+      <c r="F47" t="n">
+        <v>5808</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="1" t="inlineStr">
         <is>
           <t>Item</t>
         </is>
       </c>
-      <c r="B48" s="1" t="inlineStr">
+      <c r="B49" s="1" t="inlineStr">
         <is>
           <t>Provisional sums (partners, until quotes due 12:00 pm Wed 28/10/2026)</t>
         </is>
       </c>
-      <c r="C48" s="1" t="inlineStr">
+      <c r="C49" s="1" t="inlineStr">
         <is>
           <t>Allowance</t>
         </is>
       </c>
-      <c r="D48" s="1" t="inlineStr"/>
-      <c r="E48" s="1" t="inlineStr">
+      <c r="D49" s="1" t="inlineStr"/>
+      <c r="E49" s="1" t="inlineStr">
         <is>
           <t>Mark-up</t>
         </is>
       </c>
-      <c r="F48" s="1" t="inlineStr">
+      <c r="F49" s="1" t="inlineStr">
         <is>
           <t>Amount ex GST</t>
         </is>
       </c>
-      <c r="G48" s="1" t="n"/>
-      <c r="H48" s="1" t="n"/>
-    </row>
-    <row r="49">
-      <c r="A49" t="inlineStr">
-        <is>
-          <t>PS1</t>
-        </is>
-      </c>
-      <c r="B49" t="inlineStr">
-        <is>
-          <t>Road imaging partner: vehicle-mounted imaging of the network (with roadside) and sealed/unsealed road rating: 1,110 km x $90 + 1,890 km x $55 + $28,000 mobilisation and outputs</t>
-        </is>
-      </c>
-      <c r="C49" t="n">
-        <v>231850</v>
-      </c>
-      <c r="D49" t="inlineStr"/>
-      <c r="E49" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="F49">
-        <f>C49*(1+E49)</f>
-        <v/>
-      </c>
+      <c r="G49" s="1" t="n"/>
+      <c r="H49" s="1" t="n"/>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>PS2</t>
+          <t>PS1</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Bridge partner: Level 2, 127 structures</t>
+          <t>Road imaging partner: vehicle-mounted imaging of the network (with roadside) and sealed/unsealed road rating: 1,110 km x $90 + 1,890 km x $55 + $28,000 mobilisation and outputs</t>
         </is>
       </c>
       <c r="C50" t="n">
-        <v>117400</v>
+        <v>231850</v>
       </c>
       <c r="D50" t="inlineStr"/>
       <c r="E50" t="n">
@@ -1820,16 +1811,16 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>PS3</t>
+          <t>PS2</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Valuer: review and signed report</t>
+          <t>Bridge partner: Level 2, 127 structures</t>
         </is>
       </c>
       <c r="C51" t="n">
-        <v>30000</v>
+        <v>117400</v>
       </c>
       <c r="D51" t="inlineStr"/>
       <c r="E51" t="n">
@@ -1843,16 +1834,16 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>PS3b</t>
+          <t>PS3</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Valuer: valuation calculations and benchmark unit rates</t>
+          <t>Valuer: review and signed report</t>
         </is>
       </c>
       <c r="C52" t="n">
-        <v>18000</v>
+        <v>30000</v>
       </c>
       <c r="D52" t="inlineStr"/>
       <c r="E52" t="n">
@@ -1863,26 +1854,49 @@
         <v/>
       </c>
     </row>
-    <row r="54">
-      <c r="A54" s="2" t="inlineStr"/>
-      <c r="B54" s="2" t="inlineStr">
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>PS3b</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>Valuer: valuation calculations and benchmark unit rates</t>
+        </is>
+      </c>
+      <c r="C53" t="n">
+        <v>18000</v>
+      </c>
+      <c r="D53" t="inlineStr"/>
+      <c r="E53" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="F53">
+        <f>C53*(1+E53)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="2" t="inlineStr"/>
+      <c r="B55" s="2" t="inlineStr">
         <is>
           <t>Year 1 total ex GST</t>
         </is>
       </c>
-      <c r="C54" s="2" t="inlineStr"/>
-      <c r="D54" s="2" t="inlineStr"/>
-      <c r="E54" s="2" t="inlineStr"/>
-      <c r="F54" s="2">
-        <f>F36+SUM(F39:F40)+SUM(F43:F46)+SUM(F49:F52)</f>
-        <v/>
-      </c>
-      <c r="G54" s="2" t="n"/>
-      <c r="H54" s="2" t="n"/>
-    </row>
-    <row r="55">
-      <c r="A55" t="inlineStr"/>
-      <c r="B55" t="inlineStr">
+      <c r="C55" s="2" t="inlineStr"/>
+      <c r="D55" s="2" t="inlineStr"/>
+      <c r="E55" s="2" t="inlineStr"/>
+      <c r="F55" s="2">
+        <f>F36+SUM(F39:F40)+SUM(F43:F47)+SUM(F50:F53)</f>
+        <v/>
+      </c>
+      <c r="G55" s="2" t="n"/>
+      <c r="H55" s="2" t="n"/>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr"/>
+      <c r="B56" t="inlineStr">
         <is>
           <t>Removed from Rev F: PS1 point-asset, kerb and footpath rating ($71,425), PS1 mobilisation reduced by $7,000, PS1k GIS/register $20,500 (now JCE), B3 field verification and E2 travel (replaced by drone campaigns)</t>
         </is>
@@ -1944,7 +1958,7 @@
         </is>
       </c>
       <c r="C2">
-        <f>'Year 1 Rev G'!F54</f>
+        <f>'Year 1 Rev G'!F55</f>
         <v/>
       </c>
       <c r="D2">
@@ -1968,7 +1982,7 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>195380</v>
+        <v>196880</v>
       </c>
       <c r="D3">
         <f>C3*0.1</f>
@@ -1991,7 +2005,7 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>207720</v>
+        <v>209260</v>
       </c>
       <c r="D4">
         <f>C4*0.1</f>
@@ -2014,7 +2028,7 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>167500</v>
+        <v>169090</v>
       </c>
       <c r="D5">
         <f>C5*0.1</f>
@@ -2037,7 +2051,7 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>254390</v>
+        <v>256020</v>
       </c>
       <c r="D6">
         <f>C6*0.1</f>
@@ -2125,7 +2139,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>173736.12</v>
+        <v>175260.3</v>
       </c>
     </row>
     <row r="3">
@@ -2135,7 +2149,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>180779.47</v>
+        <v>182365.45</v>
       </c>
     </row>
     <row r="4">
@@ -2145,7 +2159,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>9182.450000000001</v>
+        <v>9263.01</v>
       </c>
     </row>
     <row r="5">
@@ -2155,7 +2169,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>23147.42</v>
+        <v>23350.5</v>
       </c>
     </row>
     <row r="6">
@@ -2165,7 +2179,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>6495.54</v>
+        <v>6552.52</v>
       </c>
     </row>
     <row r="7">
@@ -2175,7 +2189,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>13147.6</v>
+        <v>13262.94</v>
       </c>
     </row>
     <row r="8">
@@ -2185,7 +2199,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>48677.42</v>
+        <v>49104.46</v>
       </c>
     </row>
     <row r="9">
@@ -2195,7 +2209,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>21738.75</v>
+        <v>21929.47</v>
       </c>
     </row>
     <row r="10">
@@ -2205,7 +2219,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>1826.06</v>
+        <v>1842.08</v>
       </c>
     </row>
     <row r="11">
@@ -2215,7 +2229,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>171127.47</v>
+        <v>172628.77</v>
       </c>
     </row>
     <row r="12">
@@ -2225,7 +2239,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>12173.7</v>
+        <v>12280.5</v>
       </c>
     </row>
     <row r="13">

</xml_diff>